<commit_message>
formulas-queries-charts SESSION-02: checkpoint 3 — chart-bearing demo corpus
</commit_message>
<xml_diff>
--- a/tests/fixtures/workbooks/ooxml/fieldwork-q3.xlsx
+++ b/tests/fixtures/workbooks/ooxml/fieldwork-q3.xlsx
@@ -6870,8 +6870,71 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <c:chart/>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:r>
+              <a:t>Quoted by status</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Jobs!$E$1</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>Jobs!$D$2:$D$61</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Jobs!$E$2:$E$61</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="100"/>
+        <c:axId val="200"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="100"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:crossAx val="200"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="200"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:crossAx val="100"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
 </c:chartSpace>
 </file>
 

</xml_diff>